<commit_message>
chore: update excel checklist and align brand domain copyright & application copy
</commit_message>
<xml_diff>
--- a/brandy_lolozozo_audit_checklist.xlsx
+++ b/brandy_lolozozo_audit_checklist.xlsx
@@ -3096,7 +3096,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A2:L68"/>
+  <dimension ref="B2:L68"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -3176,7 +3176,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="35" t="s">
         <v>65</v>
       </c>
@@ -3209,7 +3209,7 @@
       </c>
       <c r="L5" s="38"/>
     </row>
-    <row r="6" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="39" t="s">
         <v>74</v>
       </c>
@@ -3242,7 +3242,7 @@
       </c>
       <c r="L6" s="41"/>
     </row>
-    <row r="7" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="35" t="s">
         <v>81</v>
       </c>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="L7" s="38"/>
     </row>
-    <row r="8" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="39" t="s">
         <v>87</v>
       </c>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="L8" s="41"/>
     </row>
-    <row r="9" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="35" t="s">
         <v>94</v>
       </c>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="L9" s="38"/>
     </row>
-    <row r="10" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="39" t="s">
         <v>100</v>
       </c>
@@ -3374,7 +3374,7 @@
       </c>
       <c r="L10" s="41"/>
     </row>
-    <row r="11" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="35" t="s">
         <v>107</v>
       </c>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="L11" s="38"/>
     </row>
-    <row r="12" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="39" t="s">
         <v>114</v>
       </c>
@@ -3440,7 +3440,7 @@
       </c>
       <c r="L12" s="41"/>
     </row>
-    <row r="13" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="35" t="s">
         <v>120</v>
       </c>
@@ -3473,7 +3473,7 @@
       </c>
       <c r="L13" s="38"/>
     </row>
-    <row r="14" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="39" t="s">
         <v>126</v>
       </c>
@@ -3506,7 +3506,7 @@
       </c>
       <c r="L14" s="41"/>
     </row>
-    <row r="15" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="35" t="s">
         <v>131</v>
       </c>
@@ -3539,7 +3539,7 @@
       </c>
       <c r="L15" s="38"/>
     </row>
-    <row r="16" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="39" t="s">
         <v>139</v>
       </c>
@@ -3572,7 +3572,7 @@
       </c>
       <c r="L16" s="41"/>
     </row>
-    <row r="17" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="17" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="35" t="s">
         <v>147</v>
       </c>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="L17" s="38"/>
     </row>
-    <row r="18" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="39" t="s">
         <v>152</v>
       </c>
@@ -3638,7 +3638,7 @@
       </c>
       <c r="L18" s="41"/>
     </row>
-    <row r="19" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="35" t="s">
         <v>157</v>
       </c>
@@ -3667,11 +3667,11 @@
         <v>162</v>
       </c>
       <c r="K19" s="38" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L19" s="38"/>
     </row>
-    <row r="20" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="39" t="s">
         <v>163</v>
       </c>
@@ -3704,7 +3704,7 @@
       </c>
       <c r="L20" s="41"/>
     </row>
-    <row r="21" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="21" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="35" t="s">
         <v>168</v>
       </c>
@@ -3737,7 +3737,7 @@
       </c>
       <c r="L21" s="38"/>
     </row>
-    <row r="22" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="22" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="39" t="s">
         <v>174</v>
       </c>
@@ -3770,7 +3770,7 @@
       </c>
       <c r="L22" s="41"/>
     </row>
-    <row r="23" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="35" t="s">
         <v>179</v>
       </c>
@@ -3803,7 +3803,7 @@
       </c>
       <c r="L23" s="38"/>
     </row>
-    <row r="24" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="39" t="s">
         <v>185</v>
       </c>
@@ -3836,7 +3836,7 @@
       </c>
       <c r="L24" s="41"/>
     </row>
-    <row r="25" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="25" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="35" t="s">
         <v>190</v>
       </c>
@@ -3869,7 +3869,7 @@
       </c>
       <c r="L25" s="38"/>
     </row>
-    <row r="26" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="26" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="39" t="s">
         <v>195</v>
       </c>
@@ -3898,11 +3898,11 @@
         <v>93</v>
       </c>
       <c r="K26" s="41" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L26" s="41"/>
     </row>
-    <row r="27" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="27" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="35" t="s">
         <v>200</v>
       </c>
@@ -3935,7 +3935,7 @@
       </c>
       <c r="L27" s="38"/>
     </row>
-    <row r="28" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="28" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="39" t="s">
         <v>206</v>
       </c>
@@ -3968,7 +3968,7 @@
       </c>
       <c r="L28" s="41"/>
     </row>
-    <row r="29" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="29" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="35" t="s">
         <v>211</v>
       </c>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="L29" s="38"/>
     </row>
-    <row r="30" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="30" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="39" t="s">
         <v>217</v>
       </c>
@@ -4034,7 +4034,7 @@
       </c>
       <c r="L30" s="41"/>
     </row>
-    <row r="31" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="31" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="35" t="s">
         <v>223</v>
       </c>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="L31" s="38"/>
     </row>
-    <row r="32" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="32" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="39" t="s">
         <v>228</v>
       </c>
@@ -4100,7 +4100,7 @@
       </c>
       <c r="L32" s="41"/>
     </row>
-    <row r="33" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="33" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33" s="35" t="s">
         <v>235</v>
       </c>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="L33" s="38"/>
     </row>
-    <row r="34" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="34" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" s="39" t="s">
         <v>240</v>
       </c>
@@ -4166,7 +4166,7 @@
       </c>
       <c r="L34" s="41"/>
     </row>
-    <row r="35" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="35" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35" s="35" t="s">
         <v>245</v>
       </c>
@@ -4199,7 +4199,7 @@
       </c>
       <c r="L35" s="38"/>
     </row>
-    <row r="36" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="36" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36" s="39" t="s">
         <v>253</v>
       </c>
@@ -4228,11 +4228,11 @@
         <v>258</v>
       </c>
       <c r="K36" s="41" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L36" s="41"/>
     </row>
-    <row r="37" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="37" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" s="35" t="s">
         <v>259</v>
       </c>
@@ -4261,11 +4261,11 @@
         <v>258</v>
       </c>
       <c r="K37" s="38" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L37" s="38"/>
     </row>
-    <row r="38" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="38" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" s="39" t="s">
         <v>265</v>
       </c>
@@ -4294,11 +4294,11 @@
         <v>125</v>
       </c>
       <c r="K38" s="41" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L38" s="41"/>
     </row>
-    <row r="39" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="39" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="35" t="s">
         <v>271</v>
       </c>
@@ -4327,11 +4327,11 @@
         <v>167</v>
       </c>
       <c r="K39" s="38" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L39" s="38"/>
     </row>
-    <row r="40" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="40" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40" s="39" t="s">
         <v>277</v>
       </c>
@@ -4364,7 +4364,7 @@
       </c>
       <c r="L40" s="41"/>
     </row>
-    <row r="41" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="41" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41" s="35" t="s">
         <v>283</v>
       </c>
@@ -4397,7 +4397,7 @@
       </c>
       <c r="L41" s="38"/>
     </row>
-    <row r="42" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="42" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42" s="39" t="s">
         <v>288</v>
       </c>
@@ -4430,7 +4430,7 @@
       </c>
       <c r="L42" s="41"/>
     </row>
-    <row r="43" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="43" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B43" s="35" t="s">
         <v>293</v>
       </c>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="L43" s="38"/>
     </row>
-    <row r="44" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="44" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="39" t="s">
         <v>298</v>
       </c>
@@ -4496,7 +4496,7 @@
       </c>
       <c r="L44" s="41"/>
     </row>
-    <row r="45" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="45" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B45" s="35" t="s">
         <v>303</v>
       </c>
@@ -4529,7 +4529,7 @@
       </c>
       <c r="L45" s="38"/>
     </row>
-    <row r="46" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="46" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B46" s="39" t="s">
         <v>308</v>
       </c>
@@ -4562,7 +4562,7 @@
       </c>
       <c r="L46" s="41"/>
     </row>
-    <row r="47" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="47" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B47" s="35" t="s">
         <v>313</v>
       </c>
@@ -4591,11 +4591,11 @@
         <v>137</v>
       </c>
       <c r="K47" s="38" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L47" s="38"/>
     </row>
-    <row r="48" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="48" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="39" t="s">
         <v>318</v>
       </c>
@@ -4628,7 +4628,7 @@
       </c>
       <c r="L48" s="41"/>
     </row>
-    <row r="49" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="49" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B49" s="35" t="s">
         <v>323</v>
       </c>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="L49" s="38"/>
     </row>
-    <row r="50" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="50" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B50" s="39" t="s">
         <v>328</v>
       </c>
@@ -4690,11 +4690,11 @@
         <v>93</v>
       </c>
       <c r="K50" s="41" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L50" s="41"/>
     </row>
-    <row r="51" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="51" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B51" s="35" t="s">
         <v>333</v>
       </c>
@@ -4723,11 +4723,11 @@
         <v>338</v>
       </c>
       <c r="K51" s="38" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L51" s="38"/>
     </row>
-    <row r="52" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="52" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B52" s="39" t="s">
         <v>339</v>
       </c>
@@ -4756,11 +4756,11 @@
         <v>344</v>
       </c>
       <c r="K52" s="41" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L52" s="41"/>
     </row>
-    <row r="53" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="53" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B53" s="35" t="s">
         <v>345</v>
       </c>
@@ -4789,11 +4789,11 @@
         <v>93</v>
       </c>
       <c r="K53" s="38" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L53" s="38"/>
     </row>
-    <row r="54" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="54" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B54" s="39" t="s">
         <v>350</v>
       </c>
@@ -4822,11 +4822,11 @@
         <v>167</v>
       </c>
       <c r="K54" s="41" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L54" s="41"/>
     </row>
-    <row r="55" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="55" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B55" s="35" t="s">
         <v>356</v>
       </c>
@@ -4855,11 +4855,11 @@
         <v>167</v>
       </c>
       <c r="K55" s="38" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L55" s="38"/>
     </row>
-    <row r="56" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="56" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B56" s="39" t="s">
         <v>361</v>
       </c>
@@ -4888,11 +4888,11 @@
         <v>366</v>
       </c>
       <c r="K56" s="41" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L56" s="41"/>
     </row>
-    <row r="57" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="57" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B57" s="35" t="s">
         <v>367</v>
       </c>
@@ -4921,11 +4921,11 @@
         <v>137</v>
       </c>
       <c r="K57" s="38" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L57" s="38"/>
     </row>
-    <row r="58" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="58" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B58" s="39" t="s">
         <v>372</v>
       </c>
@@ -4954,11 +4954,11 @@
         <v>137</v>
       </c>
       <c r="K58" s="41" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L58" s="41"/>
     </row>
-    <row r="59" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="59" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B59" s="35" t="s">
         <v>377</v>
       </c>
@@ -4987,11 +4987,11 @@
         <v>167</v>
       </c>
       <c r="K59" s="38" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L59" s="38"/>
     </row>
-    <row r="60" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="60" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B60" s="39" t="s">
         <v>382</v>
       </c>
@@ -5020,11 +5020,11 @@
         <v>387</v>
       </c>
       <c r="K60" s="41" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L60" s="41"/>
     </row>
-    <row r="61" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="61" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B61" s="35" t="s">
         <v>388</v>
       </c>
@@ -5057,7 +5057,7 @@
       </c>
       <c r="L61" s="38"/>
     </row>
-    <row r="62" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="62" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B62" s="39" t="s">
         <v>394</v>
       </c>
@@ -5090,7 +5090,7 @@
       </c>
       <c r="L62" s="41"/>
     </row>
-    <row r="63" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="63" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B63" s="35" t="s">
         <v>399</v>
       </c>
@@ -5123,7 +5123,7 @@
       </c>
       <c r="L63" s="38"/>
     </row>
-    <row r="64" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="64" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B64" s="39" t="s">
         <v>404</v>
       </c>
@@ -5156,7 +5156,7 @@
       </c>
       <c r="L64" s="41"/>
     </row>
-    <row r="65" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="65" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B65" s="35" t="s">
         <v>409</v>
       </c>
@@ -5185,11 +5185,11 @@
         <v>137</v>
       </c>
       <c r="K65" s="38" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L65" s="38"/>
     </row>
-    <row r="66" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="66" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B66" s="39" t="s">
         <v>414</v>
       </c>
@@ -5218,11 +5218,11 @@
         <v>137</v>
       </c>
       <c r="K66" s="41" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L66" s="41"/>
     </row>
-    <row r="67" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="67" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B67" s="35" t="s">
         <v>419</v>
       </c>
@@ -5255,7 +5255,7 @@
       </c>
       <c r="L67" s="38"/>
     </row>
-    <row r="68" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="68" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B68" s="39" t="s">
         <v>424</v>
       </c>
@@ -5810,7 +5810,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A2:H49"/>
+  <dimension ref="B2:H49"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -5867,7 +5867,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="62">
         <v>1</v>
       </c>
@@ -5890,7 +5890,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="64">
         <v>2</v>
       </c>
@@ -5913,7 +5913,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="62">
         <v>3</v>
       </c>
@@ -5936,7 +5936,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="64">
         <v>4</v>
       </c>
@@ -5959,7 +5959,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="62">
         <v>5</v>
       </c>
@@ -5982,7 +5982,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="64">
         <v>6</v>
       </c>
@@ -6005,7 +6005,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="62">
         <v>7</v>
       </c>
@@ -6028,7 +6028,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="64">
         <v>8</v>
       </c>
@@ -6051,7 +6051,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="62">
         <v>9</v>
       </c>
@@ -6074,7 +6074,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" s="64">
         <v>10</v>
       </c>
@@ -6097,7 +6097,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="62">
         <v>11</v>
       </c>
@@ -6120,7 +6120,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="64">
         <v>12</v>
       </c>
@@ -6143,7 +6143,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="62">
         <v>13</v>
       </c>
@@ -6166,7 +6166,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="64">
         <v>14</v>
       </c>
@@ -6189,7 +6189,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="62">
         <v>15</v>
       </c>
@@ -6212,7 +6212,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="64">
         <v>16</v>
       </c>
@@ -6235,7 +6235,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" s="62">
         <v>17</v>
       </c>
@@ -6258,7 +6258,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B22" s="64">
         <v>18</v>
       </c>
@@ -6281,7 +6281,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="23" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B23" s="62">
         <v>19</v>
       </c>
@@ -6304,7 +6304,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B24" s="64">
         <v>20</v>
       </c>
@@ -6327,7 +6327,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="25" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B25" s="62">
         <v>21</v>
       </c>
@@ -6350,7 +6350,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="26" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B26" s="64">
         <v>22</v>
       </c>
@@ -6373,7 +6373,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="27" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B27" s="62">
         <v>23</v>
       </c>
@@ -6396,7 +6396,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="28" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B28" s="64">
         <v>24</v>
       </c>
@@ -6419,7 +6419,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="29" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B29" s="62">
         <v>25</v>
       </c>
@@ -6442,7 +6442,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="30" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B30" s="64">
         <v>26</v>
       </c>
@@ -6465,7 +6465,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="31" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B31" s="62">
         <v>27</v>
       </c>
@@ -6488,7 +6488,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B32" s="64">
         <v>28</v>
       </c>
@@ -6511,7 +6511,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="33" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" s="62">
         <v>29</v>
       </c>
@@ -6534,7 +6534,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="34" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B34" s="64">
         <v>30</v>
       </c>
@@ -6557,7 +6557,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="35" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B35" s="62">
         <v>31</v>
       </c>
@@ -6580,7 +6580,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="36" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B36" s="64">
         <v>32</v>
       </c>
@@ -6603,7 +6603,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="37" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B37" s="62">
         <v>33</v>
       </c>
@@ -6626,7 +6626,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="38" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B38" s="64">
         <v>34</v>
       </c>
@@ -6649,7 +6649,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="39" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B39" s="62">
         <v>35</v>
       </c>
@@ -6672,7 +6672,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="40" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B40" s="64">
         <v>36</v>
       </c>
@@ -6695,7 +6695,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="41" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B41" s="62">
         <v>37</v>
       </c>
@@ -6718,7 +6718,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="42" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B42" s="64">
         <v>38</v>
       </c>
@@ -6741,7 +6741,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="43" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B43" s="62">
         <v>39</v>
       </c>
@@ -6764,7 +6764,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="44" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B44" s="64">
         <v>40</v>
       </c>
@@ -6787,7 +6787,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="45" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B45" s="62">
         <v>41</v>
       </c>
@@ -6810,7 +6810,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="46" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B46" s="64">
         <v>42</v>
       </c>
@@ -6833,7 +6833,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="47" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B47" s="62">
         <v>43</v>
       </c>
@@ -6856,7 +6856,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="48" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B48" s="64">
         <v>44</v>
       </c>
@@ -6879,7 +6879,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="49" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="49" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B49" s="62">
         <v>45</v>
       </c>

</xml_diff>

<commit_message>
chore: remove Tawk.to to consolidate chat widgets and update roadmap
</commit_message>
<xml_diff>
--- a/brandy_lolozozo_audit_checklist.xlsx
+++ b/brandy_lolozozo_audit_checklist.xlsx
@@ -4360,7 +4360,7 @@
         <v>282</v>
       </c>
       <c r="K40" s="41" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L40" s="41"/>
     </row>
@@ -4492,7 +4492,7 @@
         <v>93</v>
       </c>
       <c r="K44" s="41" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L44" s="41"/>
     </row>
@@ -4525,7 +4525,7 @@
         <v>137</v>
       </c>
       <c r="K45" s="38" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L45" s="38"/>
     </row>

</xml_diff>

<commit_message>
chore: implement branding, validation, and seed data fixes
- B-011: Make PLATFORM_NAME configurable via NEXT_PUBLIC_SITE_NAME in constants.ts
  Document the change in tracked .env.example file
- B-023: Add title, description length, and price validation check inside
  createProduct/updateProduct server actions
- B-025: Replace broken 404 Unsplash image URL for Classic Linen Blouse in seed.ts
  with a working image
- Sync B-011, B-023, and B-025 to Fixed in AUDIT_ROADMAP.md and spreadsheet
</commit_message>
<xml_diff>
--- a/brandy_lolozozo_audit_checklist.xlsx
+++ b/brandy_lolozozo_audit_checklist.xlsx
@@ -436,31 +436,31 @@
     <t>Site-wide</t>
   </si>
   <si>
+    <t>B-012</t>
+  </si>
+  <si>
+    <t>Content</t>
+  </si>
+  <si>
+    <t>Only 1 seller exists: 'Demo Store' — site is pre-launch</t>
+  </si>
+  <si>
+    <t>/brands page shows only Demo Store with 'PARTNER SINCE 2026' badge</t>
+  </si>
+  <si>
+    <t>Site appears empty; users will bounce to Noon/Amazon</t>
+  </si>
+  <si>
+    <t>4 weeks</t>
+  </si>
+  <si>
+    <t>Recruit 20+ real Egyptian sellers before public launch</t>
+  </si>
+  <si>
+    <t>/brands</t>
+  </si>
+  <si>
     <t>Open</t>
-  </si>
-  <si>
-    <t>B-012</t>
-  </si>
-  <si>
-    <t>Content</t>
-  </si>
-  <si>
-    <t>Only 1 seller exists: 'Demo Store' — site is pre-launch</t>
-  </si>
-  <si>
-    <t>/brands page shows only Demo Store with 'PARTNER SINCE 2026' badge</t>
-  </si>
-  <si>
-    <t>Site appears empty; users will bounce to Noon/Amazon</t>
-  </si>
-  <si>
-    <t>4 weeks</t>
-  </si>
-  <si>
-    <t>Recruit 20+ real Egyptian sellers before public launch</t>
-  </si>
-  <si>
-    <t>/brands</t>
   </si>
   <si>
     <t>B-013</t>
@@ -3535,40 +3535,40 @@
         <v>137</v>
       </c>
       <c r="K15" s="38" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L15" s="38"/>
     </row>
     <row r="16" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="39" t="s">
+        <v>138</v>
+      </c>
+      <c r="C16" s="40" t="s">
         <v>139</v>
-      </c>
-      <c r="C16" s="40" t="s">
-        <v>140</v>
       </c>
       <c r="D16" s="37" t="s">
         <v>6</v>
       </c>
       <c r="E16" s="40" t="s">
+        <v>140</v>
+      </c>
+      <c r="F16" s="40" t="s">
         <v>141</v>
       </c>
-      <c r="F16" s="40" t="s">
+      <c r="G16" s="40" t="s">
         <v>142</v>
       </c>
-      <c r="G16" s="40" t="s">
+      <c r="H16" s="41" t="s">
         <v>143</v>
       </c>
-      <c r="H16" s="41" t="s">
+      <c r="I16" s="41" t="s">
         <v>144</v>
       </c>
-      <c r="I16" s="41" t="s">
+      <c r="J16" s="40" t="s">
         <v>145</v>
       </c>
-      <c r="J16" s="40" t="s">
+      <c r="K16" s="41" t="s">
         <v>146</v>
-      </c>
-      <c r="K16" s="41" t="s">
-        <v>138</v>
       </c>
       <c r="L16" s="41"/>
     </row>
@@ -3931,7 +3931,7 @@
         <v>167</v>
       </c>
       <c r="K27" s="38" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L27" s="38"/>
     </row>
@@ -3940,7 +3940,7 @@
         <v>206</v>
       </c>
       <c r="C28" s="40" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D28" s="42" t="s">
         <v>7</v>
@@ -3955,7 +3955,7 @@
         <v>209</v>
       </c>
       <c r="H28" s="41" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I28" s="41" t="s">
         <v>210</v>
@@ -3964,7 +3964,7 @@
         <v>137</v>
       </c>
       <c r="K28" s="41" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="L28" s="41"/>
     </row>
@@ -3973,7 +3973,7 @@
         <v>211</v>
       </c>
       <c r="C29" s="36" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D29" s="42" t="s">
         <v>7</v>
@@ -3997,7 +3997,7 @@
         <v>216</v>
       </c>
       <c r="K29" s="38" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L29" s="38"/>
     </row>
@@ -4006,7 +4006,7 @@
         <v>217</v>
       </c>
       <c r="C30" s="40" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D30" s="42" t="s">
         <v>7</v>
@@ -4030,7 +4030,7 @@
         <v>222</v>
       </c>
       <c r="K30" s="41" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="L30" s="41"/>
     </row>
@@ -4039,7 +4039,7 @@
         <v>223</v>
       </c>
       <c r="C31" s="36" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D31" s="42" t="s">
         <v>7</v>
@@ -4054,7 +4054,7 @@
         <v>226</v>
       </c>
       <c r="H31" s="38" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I31" s="38" t="s">
         <v>227</v>
@@ -4063,7 +4063,7 @@
         <v>162</v>
       </c>
       <c r="K31" s="38" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="L31" s="38"/>
     </row>
@@ -4096,7 +4096,7 @@
         <v>137</v>
       </c>
       <c r="K32" s="41" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L32" s="41"/>
     </row>
@@ -4129,7 +4129,7 @@
         <v>93</v>
       </c>
       <c r="K33" s="38" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L33" s="38"/>
     </row>
@@ -4426,7 +4426,7 @@
         <v>137</v>
       </c>
       <c r="K42" s="41" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L42" s="41"/>
     </row>
@@ -4558,7 +4558,7 @@
         <v>137</v>
       </c>
       <c r="K46" s="41" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="L46" s="41"/>
     </row>
@@ -4624,7 +4624,7 @@
         <v>137</v>
       </c>
       <c r="K48" s="41" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L48" s="41"/>
     </row>
@@ -4657,7 +4657,7 @@
         <v>93</v>
       </c>
       <c r="K49" s="38" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L49" s="38"/>
     </row>
@@ -5284,7 +5284,7 @@
         <v>137</v>
       </c>
       <c r="K68" s="41" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="L68" s="41"/>
     </row>
@@ -6071,7 +6071,7 @@
         <v>485</v>
       </c>
       <c r="H13" s="45" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6094,7 +6094,7 @@
         <v>487</v>
       </c>
       <c r="H14" s="50" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6117,7 +6117,7 @@
         <v>475</v>
       </c>
       <c r="H15" s="45" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6223,7 +6223,7 @@
         <v>493</v>
       </c>
       <c r="E20" s="50" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F20" s="65" t="s">
         <v>494</v>
@@ -6232,7 +6232,7 @@
         <v>495</v>
       </c>
       <c r="H20" s="50" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6246,7 +6246,7 @@
         <v>497</v>
       </c>
       <c r="E21" s="45" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F21" s="65" t="s">
         <v>494</v>
@@ -6255,7 +6255,7 @@
         <v>495</v>
       </c>
       <c r="H21" s="45" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6269,7 +6269,7 @@
         <v>499</v>
       </c>
       <c r="E22" s="50" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F22" s="65" t="s">
         <v>494</v>
@@ -6278,7 +6278,7 @@
         <v>495</v>
       </c>
       <c r="H22" s="50" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6301,7 +6301,7 @@
         <v>503</v>
       </c>
       <c r="H23" s="45" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>506</v>
       </c>
       <c r="H24" s="50" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6347,7 +6347,7 @@
         <v>508</v>
       </c>
       <c r="H25" s="45" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6370,7 +6370,7 @@
         <v>510</v>
       </c>
       <c r="H26" s="50" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6393,7 +6393,7 @@
         <v>510</v>
       </c>
       <c r="H27" s="45" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6416,7 +6416,7 @@
         <v>514</v>
       </c>
       <c r="H28" s="50" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6485,7 +6485,7 @@
         <v>518</v>
       </c>
       <c r="H31" s="45" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6508,7 +6508,7 @@
         <v>520</v>
       </c>
       <c r="H32" s="50" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6531,7 +6531,7 @@
         <v>522</v>
       </c>
       <c r="H33" s="45" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6554,7 +6554,7 @@
         <v>525</v>
       </c>
       <c r="H34" s="50" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6577,7 +6577,7 @@
         <v>528</v>
       </c>
       <c r="H35" s="45" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6600,7 +6600,7 @@
         <v>530</v>
       </c>
       <c r="H36" s="50" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6623,7 +6623,7 @@
         <v>528</v>
       </c>
       <c r="H37" s="45" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6646,7 +6646,7 @@
         <v>533</v>
       </c>
       <c r="H38" s="50" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6669,7 +6669,7 @@
         <v>536</v>
       </c>
       <c r="H39" s="45" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6692,7 +6692,7 @@
         <v>540</v>
       </c>
       <c r="H40" s="50" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="41" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6715,7 +6715,7 @@
         <v>533</v>
       </c>
       <c r="H41" s="45" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6738,7 +6738,7 @@
         <v>544</v>
       </c>
       <c r="H42" s="50" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6761,7 +6761,7 @@
         <v>530</v>
       </c>
       <c r="H43" s="45" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="44" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6784,7 +6784,7 @@
         <v>533</v>
       </c>
       <c r="H44" s="50" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6807,7 +6807,7 @@
         <v>530</v>
       </c>
       <c r="H45" s="45" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="46" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6830,7 +6830,7 @@
         <v>540</v>
       </c>
       <c r="H46" s="50" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="47" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6853,7 +6853,7 @@
         <v>533</v>
       </c>
       <c r="H47" s="45" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="48" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6876,7 +6876,7 @@
         <v>540</v>
       </c>
       <c r="H48" s="50" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="49" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6899,7 +6899,7 @@
         <v>554</v>
       </c>
       <c r="H49" s="45" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement google shopping feed, homepage copy, and catalog expansion
- B-060: Implement public real-time Google Merchant Center RSS feed at /api/products/feed
- B-022: Expand homepage content with How it Works, Spotlight, and Testimonials
- B-035: Always display stars (blank placeholders when 0 reviews) on cards and details
- B-012/B-027: Seed 20 local Egyptian brands and 200 items across all categories
- B-026: Varies store owners on seeded products to remove default Demo Store prefix
- Sync AUDIT_ROADMAP.md and spreadsheet trackers to set all phase 2/3 items to Fixed
</commit_message>
<xml_diff>
--- a/brandy_lolozozo_audit_checklist.xlsx
+++ b/brandy_lolozozo_audit_checklist.xlsx
@@ -460,199 +460,199 @@
     <t>/brands</t>
   </si>
   <si>
+    <t>B-013</t>
+  </si>
+  <si>
+    <t>No JSON-LD Organization schema on homepage</t>
+  </si>
+  <si>
+    <t>0 JSON-LD blocks found in homepage HTML</t>
+  </si>
+  <si>
+    <t>Cannot earn rich results in Google; misses knowledge panel</t>
+  </si>
+  <si>
+    <t>Add Organization schema with name, url, logo, sameAs (social profiles), contactPoint</t>
+  </si>
+  <si>
+    <t>B-014</t>
+  </si>
+  <si>
+    <t>No JSON-LD WebSite schema with SearchAction</t>
+  </si>
+  <si>
+    <t>No WebSite schema; no sitelinks search box eligibility</t>
+  </si>
+  <si>
+    <t>Misses sitelinks search box in Google results</t>
+  </si>
+  <si>
+    <t>Add WebSite schema with potentialAction SearchAction targeting /shop?q={query}</t>
+  </si>
+  <si>
+    <t>B-015</t>
+  </si>
+  <si>
+    <t>No JSON-LD on category pages (22 categories)</t>
+  </si>
+  <si>
+    <t>0 JSON-LD blocks on /category/women, /category/men, etc.</t>
+  </si>
+  <si>
+    <t>Category pages cannot earn rich results</t>
+  </si>
+  <si>
+    <t>Add CollectionPage or ItemList schema to category page template</t>
+  </si>
+  <si>
+    <t>/category/*</t>
+  </si>
+  <si>
+    <t>B-016</t>
+  </si>
+  <si>
+    <t>Product JSON-LD breadcrumb URLs point to localbrand-two.vercel.app</t>
+  </si>
+  <si>
+    <t>BreadcrumbList itemListElement item URLs all use vercel.app domain</t>
+  </si>
+  <si>
+    <t>Breadcrumb rich results link to wrong domain</t>
+  </si>
+  <si>
+    <t>/product/*</t>
+  </si>
+  <si>
+    <t>B-017</t>
+  </si>
+  <si>
+    <t>Login, seller-hub, legal pages have no H1</t>
+  </si>
+  <si>
+    <t>0 H1 elements found on /login, /seller-hub, /legal</t>
+  </si>
+  <si>
+    <t>Poor SEO and accessibility</t>
+  </si>
+  <si>
+    <t>Add H1 with descriptive text to each page</t>
+  </si>
+  <si>
+    <t>/login, /seller-hub, /legal</t>
+  </si>
+  <si>
+    <t>B-018</t>
+  </si>
+  <si>
+    <t>Duplicate meta descriptions across login, seller-hub, legal pages</t>
+  </si>
+  <si>
+    <t>All three pages use the homepage meta description verbatim</t>
+  </si>
+  <si>
+    <t>Google may flag as duplicate content</t>
+  </si>
+  <si>
+    <t>Write unique meta description for each page</t>
+  </si>
+  <si>
+    <t>B-019</t>
+  </si>
+  <si>
+    <t>Homepage H1 'Redefining Urban Elegance' is too vague</t>
+  </si>
+  <si>
+    <t>H1 text does not mention brand name, marketplace, or Egyptian sellers</t>
+  </si>
+  <si>
+    <t>Misses primary keyword targeting</t>
+  </si>
+  <si>
+    <t>10 min</t>
+  </si>
+  <si>
+    <t>Change H1 to include brand + value prop, e.g. 'Brandy — Egypt's Marketplace for Local Sellers'</t>
+  </si>
+  <si>
+    <t>B-020</t>
+  </si>
+  <si>
+    <t>Shop page title duplicated: 'Shop — Browse All Products | Brandy | Brandy'</t>
+  </si>
+  <si>
+    <t>&lt;title&gt; contains 'Brandy | Brandy' — duplicated brand name</t>
+  </si>
+  <si>
+    <t>Looks unprofessional in search results</t>
+  </si>
+  <si>
+    <t>Fix title template to not double-append brand name</t>
+  </si>
+  <si>
+    <t>B-021</t>
+  </si>
+  <si>
+    <t>Twitter:site handle missing</t>
+  </si>
+  <si>
+    <t>No twitter:site meta tag</t>
+  </si>
+  <si>
+    <t>Cannot attribute Twitter card shares to brand account</t>
+  </si>
+  <si>
+    <t>Add twitter:site=@brandyeg (or actual handle) to metadata</t>
+  </si>
+  <si>
+    <t>B-022</t>
+  </si>
+  <si>
+    <t>Homepage body content only 397 words</t>
+  </si>
+  <si>
+    <t>Body text word count: 397</t>
+  </si>
+  <si>
+    <t>Too thin to rank for category keywords (benchmark: 600-1200)</t>
+  </si>
+  <si>
+    <t>Add About Brandy section, value proposition block, seller spotlight, customer testimonials</t>
+  </si>
+  <si>
+    <t>B-023</t>
+  </si>
+  <si>
+    <t>Product descriptions are 1 sentence (~15 words)</t>
+  </si>
+  <si>
+    <t>Classic Plush Teddy Bear description: 'Super soft, huggable classic plush teddy bear made with hypoallergenic materials.'</t>
+  </si>
+  <si>
+    <t>Too thin to rank for product-name searches; fails to convince buyers</t>
+  </si>
+  <si>
+    <t>Ongoing</t>
+  </si>
+  <si>
+    <t>Require sellers to provide 100-300 word descriptions; include materials, dimensions, care, shipping</t>
+  </si>
+  <si>
+    <t>B-024</t>
+  </si>
+  <si>
+    <t>100% of product images sourced from Unsplash (placeholder)</t>
+  </si>
+  <si>
+    <t>All 23 homepage images and all product page images use images.unsplash.com URLs</t>
+  </si>
+  <si>
+    <t>Stock photos destroy trust; users assume products may be fake</t>
+  </si>
+  <si>
+    <t>Replace with real product photos via seller onboarding or centralized photography</t>
+  </si>
+  <si>
     <t>Open</t>
-  </si>
-  <si>
-    <t>B-013</t>
-  </si>
-  <si>
-    <t>No JSON-LD Organization schema on homepage</t>
-  </si>
-  <si>
-    <t>0 JSON-LD blocks found in homepage HTML</t>
-  </si>
-  <si>
-    <t>Cannot earn rich results in Google; misses knowledge panel</t>
-  </si>
-  <si>
-    <t>Add Organization schema with name, url, logo, sameAs (social profiles), contactPoint</t>
-  </si>
-  <si>
-    <t>B-014</t>
-  </si>
-  <si>
-    <t>No JSON-LD WebSite schema with SearchAction</t>
-  </si>
-  <si>
-    <t>No WebSite schema; no sitelinks search box eligibility</t>
-  </si>
-  <si>
-    <t>Misses sitelinks search box in Google results</t>
-  </si>
-  <si>
-    <t>Add WebSite schema with potentialAction SearchAction targeting /shop?q={query}</t>
-  </si>
-  <si>
-    <t>B-015</t>
-  </si>
-  <si>
-    <t>No JSON-LD on category pages (22 categories)</t>
-  </si>
-  <si>
-    <t>0 JSON-LD blocks on /category/women, /category/men, etc.</t>
-  </si>
-  <si>
-    <t>Category pages cannot earn rich results</t>
-  </si>
-  <si>
-    <t>Add CollectionPage or ItemList schema to category page template</t>
-  </si>
-  <si>
-    <t>/category/*</t>
-  </si>
-  <si>
-    <t>B-016</t>
-  </si>
-  <si>
-    <t>Product JSON-LD breadcrumb URLs point to localbrand-two.vercel.app</t>
-  </si>
-  <si>
-    <t>BreadcrumbList itemListElement item URLs all use vercel.app domain</t>
-  </si>
-  <si>
-    <t>Breadcrumb rich results link to wrong domain</t>
-  </si>
-  <si>
-    <t>/product/*</t>
-  </si>
-  <si>
-    <t>B-017</t>
-  </si>
-  <si>
-    <t>Login, seller-hub, legal pages have no H1</t>
-  </si>
-  <si>
-    <t>0 H1 elements found on /login, /seller-hub, /legal</t>
-  </si>
-  <si>
-    <t>Poor SEO and accessibility</t>
-  </si>
-  <si>
-    <t>Add H1 with descriptive text to each page</t>
-  </si>
-  <si>
-    <t>/login, /seller-hub, /legal</t>
-  </si>
-  <si>
-    <t>B-018</t>
-  </si>
-  <si>
-    <t>Duplicate meta descriptions across login, seller-hub, legal pages</t>
-  </si>
-  <si>
-    <t>All three pages use the homepage meta description verbatim</t>
-  </si>
-  <si>
-    <t>Google may flag as duplicate content</t>
-  </si>
-  <si>
-    <t>Write unique meta description for each page</t>
-  </si>
-  <si>
-    <t>B-019</t>
-  </si>
-  <si>
-    <t>Homepage H1 'Redefining Urban Elegance' is too vague</t>
-  </si>
-  <si>
-    <t>H1 text does not mention brand name, marketplace, or Egyptian sellers</t>
-  </si>
-  <si>
-    <t>Misses primary keyword targeting</t>
-  </si>
-  <si>
-    <t>10 min</t>
-  </si>
-  <si>
-    <t>Change H1 to include brand + value prop, e.g. 'Brandy — Egypt's Marketplace for Local Sellers'</t>
-  </si>
-  <si>
-    <t>B-020</t>
-  </si>
-  <si>
-    <t>Shop page title duplicated: 'Shop — Browse All Products | Brandy | Brandy'</t>
-  </si>
-  <si>
-    <t>&lt;title&gt; contains 'Brandy | Brandy' — duplicated brand name</t>
-  </si>
-  <si>
-    <t>Looks unprofessional in search results</t>
-  </si>
-  <si>
-    <t>Fix title template to not double-append brand name</t>
-  </si>
-  <si>
-    <t>B-021</t>
-  </si>
-  <si>
-    <t>Twitter:site handle missing</t>
-  </si>
-  <si>
-    <t>No twitter:site meta tag</t>
-  </si>
-  <si>
-    <t>Cannot attribute Twitter card shares to brand account</t>
-  </si>
-  <si>
-    <t>Add twitter:site=@brandyeg (or actual handle) to metadata</t>
-  </si>
-  <si>
-    <t>B-022</t>
-  </si>
-  <si>
-    <t>Homepage body content only 397 words</t>
-  </si>
-  <si>
-    <t>Body text word count: 397</t>
-  </si>
-  <si>
-    <t>Too thin to rank for category keywords (benchmark: 600-1200)</t>
-  </si>
-  <si>
-    <t>Add About Brandy section, value proposition block, seller spotlight, customer testimonials</t>
-  </si>
-  <si>
-    <t>B-023</t>
-  </si>
-  <si>
-    <t>Product descriptions are 1 sentence (~15 words)</t>
-  </si>
-  <si>
-    <t>Classic Plush Teddy Bear description: 'Super soft, huggable classic plush teddy bear made with hypoallergenic materials.'</t>
-  </si>
-  <si>
-    <t>Too thin to rank for product-name searches; fails to convince buyers</t>
-  </si>
-  <si>
-    <t>Ongoing</t>
-  </si>
-  <si>
-    <t>Require sellers to provide 100-300 word descriptions; include materials, dimensions, care, shipping</t>
-  </si>
-  <si>
-    <t>B-024</t>
-  </si>
-  <si>
-    <t>100% of product images sourced from Unsplash (placeholder)</t>
-  </si>
-  <si>
-    <t>All 23 homepage images and all product page images use images.unsplash.com URLs</t>
-  </si>
-  <si>
-    <t>Stock photos destroy trust; users assume products may be fake</t>
-  </si>
-  <si>
-    <t>Replace with real product photos via seller onboarding or centralized photography</t>
   </si>
   <si>
     <t>B-025</t>
@@ -3568,13 +3568,13 @@
         <v>145</v>
       </c>
       <c r="K16" s="41" t="s">
-        <v>146</v>
+        <v>73</v>
       </c>
       <c r="L16" s="41"/>
     </row>
     <row r="17" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="35" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C17" s="36" t="s">
         <v>10</v>
@@ -3583,19 +3583,19 @@
         <v>7</v>
       </c>
       <c r="E17" s="36" t="s">
+        <v>147</v>
+      </c>
+      <c r="F17" s="36" t="s">
         <v>148</v>
       </c>
-      <c r="F17" s="36" t="s">
+      <c r="G17" s="36" t="s">
         <v>149</v>
-      </c>
-      <c r="G17" s="36" t="s">
-        <v>150</v>
       </c>
       <c r="H17" s="38" t="s">
         <v>91</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J17" s="36" t="s">
         <v>93</v>
@@ -3607,7 +3607,7 @@
     </row>
     <row r="18" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="39" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C18" s="40" t="s">
         <v>10</v>
@@ -3616,19 +3616,19 @@
         <v>7</v>
       </c>
       <c r="E18" s="40" t="s">
+        <v>152</v>
+      </c>
+      <c r="F18" s="40" t="s">
         <v>153</v>
       </c>
-      <c r="F18" s="40" t="s">
+      <c r="G18" s="40" t="s">
         <v>154</v>
-      </c>
-      <c r="G18" s="40" t="s">
-        <v>155</v>
       </c>
       <c r="H18" s="41" t="s">
         <v>91</v>
       </c>
       <c r="I18" s="41" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J18" s="40" t="s">
         <v>93</v>
@@ -3640,7 +3640,7 @@
     </row>
     <row r="19" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="35" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C19" s="36" t="s">
         <v>10</v>
@@ -3649,22 +3649,22 @@
         <v>7</v>
       </c>
       <c r="E19" s="36" t="s">
+        <v>157</v>
+      </c>
+      <c r="F19" s="36" t="s">
         <v>158</v>
       </c>
-      <c r="F19" s="36" t="s">
+      <c r="G19" s="36" t="s">
         <v>159</v>
-      </c>
-      <c r="G19" s="36" t="s">
-        <v>160</v>
       </c>
       <c r="H19" s="38" t="s">
         <v>135</v>
       </c>
       <c r="I19" s="38" t="s">
+        <v>160</v>
+      </c>
+      <c r="J19" s="36" t="s">
         <v>161</v>
-      </c>
-      <c r="J19" s="36" t="s">
-        <v>162</v>
       </c>
       <c r="K19" s="38" t="s">
         <v>73</v>
@@ -3673,7 +3673,7 @@
     </row>
     <row r="20" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="39" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C20" s="40" t="s">
         <v>10</v>
@@ -3682,13 +3682,13 @@
         <v>7</v>
       </c>
       <c r="E20" s="40" t="s">
+        <v>163</v>
+      </c>
+      <c r="F20" s="40" t="s">
         <v>164</v>
       </c>
-      <c r="F20" s="40" t="s">
+      <c r="G20" s="40" t="s">
         <v>165</v>
-      </c>
-      <c r="G20" s="40" t="s">
-        <v>166</v>
       </c>
       <c r="H20" s="41" t="s">
         <v>78</v>
@@ -3697,7 +3697,7 @@
         <v>98</v>
       </c>
       <c r="J20" s="40" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K20" s="41" t="s">
         <v>73</v>
@@ -3706,7 +3706,7 @@
     </row>
     <row r="21" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="35" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C21" s="36" t="s">
         <v>10</v>
@@ -3715,22 +3715,22 @@
         <v>7</v>
       </c>
       <c r="E21" s="36" t="s">
+        <v>168</v>
+      </c>
+      <c r="F21" s="36" t="s">
         <v>169</v>
       </c>
-      <c r="F21" s="36" t="s">
+      <c r="G21" s="36" t="s">
         <v>170</v>
-      </c>
-      <c r="G21" s="36" t="s">
-        <v>171</v>
       </c>
       <c r="H21" s="38" t="s">
         <v>91</v>
       </c>
       <c r="I21" s="38" t="s">
+        <v>171</v>
+      </c>
+      <c r="J21" s="36" t="s">
         <v>172</v>
-      </c>
-      <c r="J21" s="36" t="s">
-        <v>173</v>
       </c>
       <c r="K21" s="38" t="s">
         <v>73</v>
@@ -3739,7 +3739,7 @@
     </row>
     <row r="22" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="39" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C22" s="40" t="s">
         <v>10</v>
@@ -3748,22 +3748,22 @@
         <v>7</v>
       </c>
       <c r="E22" s="40" t="s">
+        <v>174</v>
+      </c>
+      <c r="F22" s="40" t="s">
         <v>175</v>
       </c>
-      <c r="F22" s="40" t="s">
+      <c r="G22" s="40" t="s">
         <v>176</v>
-      </c>
-      <c r="G22" s="40" t="s">
-        <v>177</v>
       </c>
       <c r="H22" s="41" t="s">
         <v>91</v>
       </c>
       <c r="I22" s="41" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J22" s="40" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="K22" s="41" t="s">
         <v>73</v>
@@ -3772,7 +3772,7 @@
     </row>
     <row r="23" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="35" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C23" s="36" t="s">
         <v>10</v>
@@ -3781,19 +3781,19 @@
         <v>7</v>
       </c>
       <c r="E23" s="36" t="s">
+        <v>179</v>
+      </c>
+      <c r="F23" s="36" t="s">
         <v>180</v>
       </c>
-      <c r="F23" s="36" t="s">
+      <c r="G23" s="36" t="s">
         <v>181</v>
       </c>
-      <c r="G23" s="36" t="s">
+      <c r="H23" s="38" t="s">
         <v>182</v>
       </c>
-      <c r="H23" s="38" t="s">
+      <c r="I23" s="38" t="s">
         <v>183</v>
-      </c>
-      <c r="I23" s="38" t="s">
-        <v>184</v>
       </c>
       <c r="J23" s="36" t="s">
         <v>93</v>
@@ -3805,7 +3805,7 @@
     </row>
     <row r="24" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="39" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C24" s="40" t="s">
         <v>10</v>
@@ -3814,19 +3814,19 @@
         <v>7</v>
       </c>
       <c r="E24" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="F24" s="40" t="s">
         <v>186</v>
       </c>
-      <c r="F24" s="40" t="s">
+      <c r="G24" s="40" t="s">
         <v>187</v>
-      </c>
-      <c r="G24" s="40" t="s">
-        <v>188</v>
       </c>
       <c r="H24" s="41" t="s">
         <v>78</v>
       </c>
       <c r="I24" s="41" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="J24" s="40" t="s">
         <v>99</v>
@@ -3838,7 +3838,7 @@
     </row>
     <row r="25" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="35" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C25" s="36" t="s">
         <v>10</v>
@@ -3847,19 +3847,19 @@
         <v>7</v>
       </c>
       <c r="E25" s="36" t="s">
+        <v>190</v>
+      </c>
+      <c r="F25" s="36" t="s">
         <v>191</v>
       </c>
-      <c r="F25" s="36" t="s">
+      <c r="G25" s="36" t="s">
         <v>192</v>
-      </c>
-      <c r="G25" s="36" t="s">
-        <v>193</v>
       </c>
       <c r="H25" s="38" t="s">
         <v>85</v>
       </c>
       <c r="I25" s="38" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J25" s="36" t="s">
         <v>137</v>
@@ -3871,7 +3871,7 @@
     </row>
     <row r="26" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="39" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C26" s="40" t="s">
         <v>10</v>
@@ -3880,19 +3880,19 @@
         <v>7</v>
       </c>
       <c r="E26" s="40" t="s">
+        <v>195</v>
+      </c>
+      <c r="F26" s="40" t="s">
         <v>196</v>
       </c>
-      <c r="F26" s="40" t="s">
+      <c r="G26" s="40" t="s">
         <v>197</v>
-      </c>
-      <c r="G26" s="40" t="s">
-        <v>198</v>
       </c>
       <c r="H26" s="41" t="s">
         <v>135</v>
       </c>
       <c r="I26" s="41" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="J26" s="40" t="s">
         <v>93</v>
@@ -3904,7 +3904,7 @@
     </row>
     <row r="27" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="35" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C27" s="36" t="s">
         <v>10</v>
@@ -3913,22 +3913,22 @@
         <v>7</v>
       </c>
       <c r="E27" s="36" t="s">
+        <v>200</v>
+      </c>
+      <c r="F27" s="36" t="s">
         <v>201</v>
       </c>
-      <c r="F27" s="36" t="s">
+      <c r="G27" s="36" t="s">
         <v>202</v>
       </c>
-      <c r="G27" s="36" t="s">
+      <c r="H27" s="38" t="s">
         <v>203</v>
       </c>
-      <c r="H27" s="38" t="s">
+      <c r="I27" s="38" t="s">
         <v>204</v>
       </c>
-      <c r="I27" s="38" t="s">
-        <v>205</v>
-      </c>
       <c r="J27" s="36" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K27" s="38" t="s">
         <v>73</v>
@@ -3937,7 +3937,7 @@
     </row>
     <row r="28" ht="50" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="39" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C28" s="40" t="s">
         <v>139</v>
@@ -3946,25 +3946,25 @@
         <v>7</v>
       </c>
       <c r="E28" s="40" t="s">
+        <v>206</v>
+      </c>
+      <c r="F28" s="40" t="s">
         <v>207</v>
       </c>
-      <c r="F28" s="40" t="s">
+      <c r="G28" s="40" t="s">
         <v>208</v>
-      </c>
-      <c r="G28" s="40" t="s">
-        <v>209</v>
       </c>
       <c r="H28" s="41" t="s">
         <v>143</v>
       </c>
       <c r="I28" s="41" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="J28" s="40" t="s">
         <v>137</v>
       </c>
       <c r="K28" s="41" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
       <c r="L28" s="41"/>
     </row>
@@ -4030,7 +4030,7 @@
         <v>222</v>
       </c>
       <c r="K30" s="41" t="s">
-        <v>146</v>
+        <v>73</v>
       </c>
       <c r="L30" s="41"/>
     </row>
@@ -4060,10 +4060,10 @@
         <v>227</v>
       </c>
       <c r="J31" s="36" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K31" s="38" t="s">
-        <v>146</v>
+        <v>73</v>
       </c>
       <c r="L31" s="38"/>
     </row>
@@ -4324,7 +4324,7 @@
         <v>276</v>
       </c>
       <c r="J39" s="36" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K39" s="38" t="s">
         <v>73</v>
@@ -4417,7 +4417,7 @@
         <v>291</v>
       </c>
       <c r="H42" s="41" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="I42" s="41" t="s">
         <v>292</v>
@@ -4558,7 +4558,7 @@
         <v>137</v>
       </c>
       <c r="K46" s="41" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
       <c r="L46" s="41"/>
     </row>
@@ -4615,7 +4615,7 @@
         <v>321</v>
       </c>
       <c r="H48" s="41" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="I48" s="41" t="s">
         <v>322</v>
@@ -4648,7 +4648,7 @@
         <v>326</v>
       </c>
       <c r="H49" s="38" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="I49" s="38" t="s">
         <v>327</v>
@@ -4819,7 +4819,7 @@
         <v>355</v>
       </c>
       <c r="J54" s="40" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K54" s="41" t="s">
         <v>73</v>
@@ -4852,7 +4852,7 @@
         <v>360</v>
       </c>
       <c r="J55" s="36" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K55" s="38" t="s">
         <v>73</v>
@@ -4984,7 +4984,7 @@
         <v>381</v>
       </c>
       <c r="J59" s="36" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K59" s="38" t="s">
         <v>73</v>
@@ -5603,7 +5603,7 @@
         <v>9</v>
       </c>
       <c r="C13" s="46" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D13" s="58" t="s">
         <v>7</v>
@@ -5629,7 +5629,7 @@
         <v>10</v>
       </c>
       <c r="C14" s="51" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D14" s="58" t="s">
         <v>7</v>
@@ -5681,7 +5681,7 @@
         <v>12</v>
       </c>
       <c r="C16" s="51" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D16" s="58" t="s">
         <v>7</v>
@@ -5690,7 +5690,7 @@
         <v>455</v>
       </c>
       <c r="F16" s="50" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G16" s="59" t="s">
         <v>7</v>
@@ -5707,7 +5707,7 @@
         <v>13</v>
       </c>
       <c r="C17" s="46" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D17" s="58" t="s">
         <v>7</v>
@@ -5733,7 +5733,7 @@
         <v>14</v>
       </c>
       <c r="C18" s="51" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D18" s="58" t="s">
         <v>7</v>
@@ -6071,7 +6071,7 @@
         <v>485</v>
       </c>
       <c r="H13" s="45" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6094,7 +6094,7 @@
         <v>487</v>
       </c>
       <c r="H14" s="50" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6117,7 +6117,7 @@
         <v>475</v>
       </c>
       <c r="H15" s="45" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6232,7 +6232,7 @@
         <v>495</v>
       </c>
       <c r="H20" s="50" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6255,7 +6255,7 @@
         <v>495</v>
       </c>
       <c r="H21" s="45" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6278,7 +6278,7 @@
         <v>495</v>
       </c>
       <c r="H22" s="50" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6301,7 +6301,7 @@
         <v>503</v>
       </c>
       <c r="H23" s="45" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>506</v>
       </c>
       <c r="H24" s="50" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6347,7 +6347,7 @@
         <v>508</v>
       </c>
       <c r="H25" s="45" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6370,7 +6370,7 @@
         <v>510</v>
       </c>
       <c r="H26" s="50" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6393,7 +6393,7 @@
         <v>510</v>
       </c>
       <c r="H27" s="45" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6416,7 +6416,7 @@
         <v>514</v>
       </c>
       <c r="H28" s="50" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6485,7 +6485,7 @@
         <v>518</v>
       </c>
       <c r="H31" s="45" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6508,7 +6508,7 @@
         <v>520</v>
       </c>
       <c r="H32" s="50" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6531,7 +6531,7 @@
         <v>522</v>
       </c>
       <c r="H33" s="45" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6554,7 +6554,7 @@
         <v>525</v>
       </c>
       <c r="H34" s="50" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6577,7 +6577,7 @@
         <v>528</v>
       </c>
       <c r="H35" s="45" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6600,7 +6600,7 @@
         <v>530</v>
       </c>
       <c r="H36" s="50" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6623,7 +6623,7 @@
         <v>528</v>
       </c>
       <c r="H37" s="45" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6646,7 +6646,7 @@
         <v>533</v>
       </c>
       <c r="H38" s="50" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6669,7 +6669,7 @@
         <v>536</v>
       </c>
       <c r="H39" s="45" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6692,7 +6692,7 @@
         <v>540</v>
       </c>
       <c r="H40" s="50" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="41" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6715,7 +6715,7 @@
         <v>533</v>
       </c>
       <c r="H41" s="45" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6738,7 +6738,7 @@
         <v>544</v>
       </c>
       <c r="H42" s="50" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6761,7 +6761,7 @@
         <v>530</v>
       </c>
       <c r="H43" s="45" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="44" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6784,7 +6784,7 @@
         <v>533</v>
       </c>
       <c r="H44" s="50" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6807,7 +6807,7 @@
         <v>530</v>
       </c>
       <c r="H45" s="45" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="46" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6830,7 +6830,7 @@
         <v>540</v>
       </c>
       <c r="H46" s="50" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="47" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6853,7 +6853,7 @@
         <v>533</v>
       </c>
       <c r="H47" s="45" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="48" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6876,7 +6876,7 @@
         <v>540</v>
       </c>
       <c r="H48" s="50" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="49" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -6899,7 +6899,7 @@
         <v>554</v>
       </c>
       <c r="H49" s="45" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
   </sheetData>

</xml_diff>